<commit_message>
fix: refine the empirical specification, update new model result
</commit_message>
<xml_diff>
--- a/outputs/M1_baseline_liquidity_regression_detail.xlsx
+++ b/outputs/M1_baseline_liquidity_regression_detail.xlsx
@@ -40,19 +40,19 @@
     <t>Intercept</t>
   </si>
   <si>
+    <t>inflation_gdp_deflator_pct</t>
+  </si>
+  <si>
+    <t>trade_pct_gdp</t>
+  </si>
+  <si>
+    <t>ln_gdppc</t>
+  </si>
+  <si>
+    <t>xr_dep_pct</t>
+  </si>
+  <si>
     <t>broad_money_pct_gdp</t>
-  </si>
-  <si>
-    <t>inflation_gdp_deflator_pct</t>
-  </si>
-  <si>
-    <t>trade_pct_gdp</t>
-  </si>
-  <si>
-    <t>ln_gdppc</t>
-  </si>
-  <si>
-    <t>xr_dep_pct</t>
   </si>
 </sst>
 </file>
@@ -441,22 +441,22 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>29.95237668886436</v>
+        <v>29.9523766888643</v>
       </c>
       <c r="C2">
-        <v>28.23087896551034</v>
+        <v>28.23087896547804</v>
       </c>
       <c r="D2">
-        <v>1.060979246358471</v>
+        <v>1.060979246359682</v>
       </c>
       <c r="E2">
-        <v>0.291669874966787</v>
+        <v>0.2916698749662396</v>
       </c>
       <c r="F2">
-        <v>-26.16875327886729</v>
+        <v>-26.16875327880315</v>
       </c>
       <c r="G2">
-        <v>86.07350665659601</v>
+        <v>86.07350665653175</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -464,22 +464,22 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>0.06702316286551419</v>
+        <v>0.02435660518628829</v>
       </c>
       <c r="C3">
-        <v>0.05779663198719766</v>
+        <v>0.0909505039075543</v>
       </c>
       <c r="D3">
-        <v>1.159637864025715</v>
+        <v>0.2678006623365749</v>
       </c>
       <c r="E3">
-        <v>0.2494057531534364</v>
+        <v>0.7894940071525567</v>
       </c>
       <c r="F3">
-        <v>-0.04787273886724436</v>
+        <v>-0.1564470126062146</v>
       </c>
       <c r="G3">
-        <v>0.1819190645982727</v>
+        <v>0.2051602229787912</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -487,22 +487,22 @@
         <v>9</v>
       </c>
       <c r="B4">
-        <v>0.02435660518628832</v>
+        <v>-0.03112408994088772</v>
       </c>
       <c r="C4">
-        <v>0.09095050390757292</v>
+        <v>0.02133904583141472</v>
       </c>
       <c r="D4">
-        <v>0.2678006623365205</v>
+        <v>-1.458551154853782</v>
       </c>
       <c r="E4">
-        <v>0.7894940071525984</v>
+        <v>0.148331314546456</v>
       </c>
       <c r="F4">
-        <v>-0.1564470126062515</v>
+        <v>-0.0735447090776592</v>
       </c>
       <c r="G4">
-        <v>0.2051602229788282</v>
+        <v>0.01129652919588377</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -510,22 +510,22 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>-0.03112408994088765</v>
+        <v>-3.134683418078563</v>
       </c>
       <c r="C5">
-        <v>0.02133904583141751</v>
+        <v>3.632728714754249</v>
       </c>
       <c r="D5">
-        <v>-1.458551154853588</v>
+        <v>-0.8629004982802911</v>
       </c>
       <c r="E5">
-        <v>0.1483313145465091</v>
+        <v>0.3905921991430277</v>
       </c>
       <c r="F5">
-        <v>-0.07354470907766469</v>
+        <v>-10.35630909212525</v>
       </c>
       <c r="G5">
-        <v>0.01129652919588939</v>
+        <v>4.086942255968121</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -533,22 +533,22 @@
         <v>11</v>
       </c>
       <c r="B6">
-        <v>-3.134683418078571</v>
+        <v>0.01302226957839715</v>
       </c>
       <c r="C6">
-        <v>3.632728714758058</v>
+        <v>0.07728486040402653</v>
       </c>
       <c r="D6">
-        <v>-0.8629004982793884</v>
+        <v>0.1684970317643052</v>
       </c>
       <c r="E6">
-        <v>0.3905921991435211</v>
+        <v>0.8665879309322801</v>
       </c>
       <c r="F6">
-        <v>-10.35630909213283</v>
+        <v>-0.1406149480431748</v>
       </c>
       <c r="G6">
-        <v>4.086942255975686</v>
+        <v>0.1666594871999691</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -556,22 +556,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>0.01302226957839721</v>
+        <v>0.0670231628655142</v>
       </c>
       <c r="C7">
-        <v>0.07728486040406445</v>
+        <v>0.05779663198718442</v>
       </c>
       <c r="D7">
-        <v>0.1684970317642233</v>
+        <v>1.159637864025981</v>
       </c>
       <c r="E7">
-        <v>0.8665879309323445</v>
+        <v>0.2494057531533285</v>
       </c>
       <c r="F7">
-        <v>-0.1406149480432501</v>
+        <v>-0.04787273886721802</v>
       </c>
       <c r="G7">
-        <v>0.1666594872000445</v>
+        <v>0.1819190645982464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: compact the report, replace broad_money_pct_GDP with broad_money_growth, showing correct expected sign and improve variable significance
</commit_message>
<xml_diff>
--- a/outputs/M1_baseline_liquidity_regression_detail.xlsx
+++ b/outputs/M1_baseline_liquidity_regression_detail.xlsx
@@ -40,6 +40,9 @@
     <t>Intercept</t>
   </si>
   <si>
+    <t>broad_money_growth_pct</t>
+  </si>
+  <si>
     <t>inflation_gdp_deflator_pct</t>
   </si>
   <si>
@@ -50,9 +53,6 @@
   </si>
   <si>
     <t>xr_dep_pct</t>
-  </si>
-  <si>
-    <t>broad_money_pct_gdp</t>
   </si>
 </sst>
 </file>
@@ -441,22 +441,22 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>29.9523766888643</v>
+        <v>-0.7260745909341969</v>
       </c>
       <c r="C2">
-        <v>28.23087896547804</v>
+        <v>37.84589138134486</v>
       </c>
       <c r="D2">
-        <v>1.060979246359682</v>
+        <v>-0.01918503077700256</v>
       </c>
       <c r="E2">
-        <v>0.2916698749662396</v>
+        <v>0.9847157361013956</v>
       </c>
       <c r="F2">
-        <v>-26.16875327880315</v>
+        <v>-75.42826940027001</v>
       </c>
       <c r="G2">
-        <v>86.07350665653175</v>
+        <v>73.9761202184016</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -464,22 +464,22 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>0.02435660518628829</v>
+        <v>0.04596870475465203</v>
       </c>
       <c r="C3">
-        <v>0.0909505039075543</v>
+        <v>0.02774913696545765</v>
       </c>
       <c r="D3">
-        <v>0.2678006623365749</v>
+        <v>1.656581421320391</v>
       </c>
       <c r="E3">
-        <v>0.7894940071525567</v>
+        <v>0.09942721367621576</v>
       </c>
       <c r="F3">
-        <v>-0.1564470126062146</v>
+        <v>-0.008803989446080983</v>
       </c>
       <c r="G3">
-        <v>0.2051602229787912</v>
+        <v>0.100741398955385</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -487,22 +487,22 @@
         <v>9</v>
       </c>
       <c r="B4">
-        <v>-0.03112408994088772</v>
+        <v>-0.01950241809272713</v>
       </c>
       <c r="C4">
-        <v>0.02133904583141472</v>
+        <v>0.05757315214951274</v>
       </c>
       <c r="D4">
-        <v>-1.458551154853782</v>
+        <v>-0.3387415377584495</v>
       </c>
       <c r="E4">
-        <v>0.148331314546456</v>
+        <v>0.7352176185689552</v>
       </c>
       <c r="F4">
-        <v>-0.0735447090776592</v>
+        <v>-0.1331433093673985</v>
       </c>
       <c r="G4">
-        <v>0.01129652919588377</v>
+        <v>0.09413847318194421</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -510,22 +510,22 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>-3.134683418078563</v>
+        <v>-0.00138662976460258</v>
       </c>
       <c r="C5">
-        <v>3.632728714754249</v>
+        <v>0.01230506142030408</v>
       </c>
       <c r="D5">
-        <v>-0.8629004982802911</v>
+        <v>-0.1126877564637393</v>
       </c>
       <c r="E5">
-        <v>0.3905921991430277</v>
+        <v>0.9104095189206358</v>
       </c>
       <c r="F5">
-        <v>-10.35630909212525</v>
+        <v>-0.02567500194477273</v>
       </c>
       <c r="G5">
-        <v>4.086942255968121</v>
+        <v>0.02290174241556757</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -533,22 +533,22 @@
         <v>11</v>
       </c>
       <c r="B6">
-        <v>0.01302226957839715</v>
+        <v>0.2059099657592671</v>
       </c>
       <c r="C6">
-        <v>0.07728486040402653</v>
+        <v>1.528432296612507</v>
       </c>
       <c r="D6">
-        <v>0.1684970317643052</v>
+        <v>0.1347197165459204</v>
       </c>
       <c r="E6">
-        <v>0.8665879309322801</v>
+        <v>0.8929910021279697</v>
       </c>
       <c r="F6">
-        <v>-0.1406149480431748</v>
+        <v>-2.810989438827322</v>
       </c>
       <c r="G6">
-        <v>0.1666594871999691</v>
+        <v>3.222809370345857</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -556,22 +556,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>0.0670231628655142</v>
+        <v>0.01530861107447024</v>
       </c>
       <c r="C7">
-        <v>0.05779663198718442</v>
+        <v>0.0271993932711373</v>
       </c>
       <c r="D7">
-        <v>1.159637864025981</v>
+        <v>0.5628291382041604</v>
       </c>
       <c r="E7">
-        <v>0.2494057531533285</v>
+        <v>0.5742841228223883</v>
       </c>
       <c r="F7">
-        <v>-0.04787273886721802</v>
+        <v>-0.03837897034256531</v>
       </c>
       <c r="G7">
-        <v>0.1819190645982464</v>
+        <v>0.06899619249150579</v>
       </c>
     </row>
   </sheetData>

</xml_diff>